<commit_message>
Update CES analysis outputs and RMSE tables
</commit_message>
<xml_diff>
--- a/tables_and_figures/input_tables/national_errors.xlsx
+++ b/tables_and_figures/input_tables/national_errors.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -545,7 +545,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G3" t="b">
@@ -613,7 +613,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G4" t="b">
@@ -681,7 +681,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G5" t="b">
@@ -749,7 +749,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G6" t="b">
@@ -817,7 +817,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G7" t="b">
@@ -885,7 +885,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G8" t="b">
@@ -953,7 +953,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G9" t="b">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G10" t="b">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G11" t="b">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G12" t="b">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G13" t="b">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G14" t="b">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G15" t="b">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G16" t="b">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G17" t="b">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G18" t="b">
@@ -1578,7 +1578,7 @@
         <v>0</v>
       </c>
       <c r="J18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18">
         <v>52.18745796266161</v>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G19" t="b">
@@ -1646,7 +1646,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19">
         <v>52.18745796266161</v>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G20" t="b">
@@ -1714,7 +1714,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20">
         <v>52.18745796266161</v>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G21" t="b">
@@ -1782,7 +1782,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21">
         <v>52.18745796266161</v>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G22" t="b">
@@ -1850,7 +1850,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22">
         <v>87.20709012470589</v>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G23" t="b">
@@ -1918,7 +1918,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23">
         <v>87.20709012470589</v>
@@ -1973,7 +1973,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G24" t="b">
@@ -1986,7 +1986,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24">
         <v>87.20709012470589</v>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G25" t="b">
@@ -2054,7 +2054,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25">
         <v>87.20709012470589</v>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G26" t="b">
@@ -2122,7 +2122,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26">
         <v>88.86751429572016</v>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G27" t="b">
@@ -2190,7 +2190,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27">
         <v>88.86751429572016</v>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G28" t="b">
@@ -2258,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28">
         <v>88.86751429572016</v>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G29" t="b">
@@ -2326,7 +2326,7 @@
         <v>0</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K29">
         <v>88.86751429572016</v>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G30" t="b">
@@ -2394,7 +2394,7 @@
         <v>0</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30">
         <v>86.23135014450705</v>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G31" t="b">
@@ -2462,7 +2462,7 @@
         <v>0</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K31">
         <v>86.23135014450705</v>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G32" t="b">
@@ -2530,7 +2530,7 @@
         <v>0</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32">
         <v>86.23135014450705</v>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G33" t="b">
@@ -2598,7 +2598,7 @@
         <v>0</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33">
         <v>86.23135014450705</v>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G34" t="b">
@@ -2666,7 +2666,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34">
         <v>62.08476673915369</v>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G35" t="b">
@@ -2734,7 +2734,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K35">
         <v>62.08476673915369</v>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G36" t="b">
@@ -2802,7 +2802,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36">
         <v>62.08476673915369</v>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Unclassified</t>
         </is>
       </c>
       <c r="G37" t="b">
@@ -2870,7 +2870,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37">
         <v>62.08476673915369</v>
@@ -26045,7 +26045,7 @@
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G378" t="b">
@@ -26058,7 +26058,7 @@
         <v>0</v>
       </c>
       <c r="J378" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K378">
         <v>57.1867220532585</v>
@@ -26113,7 +26113,7 @@
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G379" t="b">
@@ -26126,7 +26126,7 @@
         <v>0</v>
       </c>
       <c r="J379" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K379">
         <v>57.1867220532585</v>
@@ -26181,7 +26181,7 @@
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G380" t="b">
@@ -26194,7 +26194,7 @@
         <v>0</v>
       </c>
       <c r="J380" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K380">
         <v>57.1867220532585</v>
@@ -26249,7 +26249,7 @@
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G381" t="b">
@@ -26262,7 +26262,7 @@
         <v>0</v>
       </c>
       <c r="J381" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K381">
         <v>57.1867220532585</v>

</xml_diff>

<commit_message>
Split figuresHQ into paper and additional notebooks; output/ subfolders; repo cleanup
- figuresHQ.ipynb builds only what the paper loads, in paper order with current table/figure numbers; additionalFiguresHQ.ipynb holds dropped exhibits, side outputs and Part II
- Outputs go to output/main, output/supplementary and output/additional; prose_numbers.tex stays at output/; .tex paths updated
- Remove excluded_work/ and the unchosen process-diagram versions (va.py, vb.py); make.py builds Version C only
- Update README.md and code/README.md
</commit_message>
<xml_diff>
--- a/tables_and_figures/input_tables/national_errors.xlsx
+++ b/tables_and_figures/input_tables/national_errors.xlsx
@@ -2398,7 +2398,7 @@
         <v>1</v>
       </c>
       <c r="K34">
-        <v>62.08476673915371</v>
+        <v>58.53764797567101</v>
       </c>
       <c r="L34">
         <v>10.21307356029052</v>
@@ -2419,7 +2419,7 @@
         <v>24</v>
       </c>
       <c r="S34">
-        <v>-51.87169317886319</v>
+        <v>-48.32457441538048</v>
       </c>
     </row>
     <row r="35" spans="1:19">
@@ -2454,7 +2454,7 @@
         <v>1</v>
       </c>
       <c r="K35">
-        <v>62.08476673915371</v>
+        <v>58.53764797567101</v>
       </c>
       <c r="L35">
         <v>10.21307356029052</v>
@@ -2475,7 +2475,7 @@
         <v>25</v>
       </c>
       <c r="S35">
-        <v>-48.37189542905355</v>
+        <v>-44.82477666557084</v>
       </c>
     </row>
     <row r="36" spans="1:19">
@@ -2510,7 +2510,7 @@
         <v>1</v>
       </c>
       <c r="K36">
-        <v>62.08476673915371</v>
+        <v>58.53764797567101</v>
       </c>
       <c r="L36">
         <v>10.21307356029052</v>
@@ -2531,7 +2531,7 @@
         <v>26</v>
       </c>
       <c r="S36">
-        <v>-48.75005182672324</v>
+        <v>-45.20293306324054</v>
       </c>
     </row>
     <row r="37" spans="1:19">
@@ -2566,7 +2566,7 @@
         <v>1</v>
       </c>
       <c r="K37">
-        <v>62.08476673915371</v>
+        <v>58.53764797567101</v>
       </c>
       <c r="L37">
         <v>10.21307356029052</v>
@@ -2587,7 +2587,7 @@
         <v>27</v>
       </c>
       <c r="S37">
-        <v>-48.68608362552613</v>
+        <v>-45.13896486204343</v>
       </c>
     </row>
     <row r="38" spans="1:19">
@@ -4638,7 +4638,7 @@
         <v>0</v>
       </c>
       <c r="K74">
-        <v>57.3909499335277</v>
+        <v>62.6433899163336</v>
       </c>
       <c r="L74">
         <v>89.80584340279077</v>
@@ -4659,7 +4659,7 @@
         <v>24</v>
       </c>
       <c r="S74">
-        <v>32.41489346926306</v>
+        <v>27.16245348645716</v>
       </c>
     </row>
     <row r="75" spans="1:19">
@@ -4694,7 +4694,7 @@
         <v>0</v>
       </c>
       <c r="K75">
-        <v>57.3909499335277</v>
+        <v>62.6433899163336</v>
       </c>
       <c r="L75">
         <v>89.80584340279077</v>
@@ -4715,7 +4715,7 @@
         <v>25</v>
       </c>
       <c r="S75">
-        <v>27.62128691766935</v>
+        <v>22.36884693486345</v>
       </c>
     </row>
     <row r="76" spans="1:19">
@@ -4750,7 +4750,7 @@
         <v>0</v>
       </c>
       <c r="K76">
-        <v>57.3909499335277</v>
+        <v>62.6433899163336</v>
       </c>
       <c r="L76">
         <v>89.80584340279077</v>
@@ -4771,7 +4771,7 @@
         <v>26</v>
       </c>
       <c r="S76">
-        <v>31.26779481350348</v>
+        <v>26.01535483069758</v>
       </c>
     </row>
     <row r="77" spans="1:19">
@@ -4806,7 +4806,7 @@
         <v>0</v>
       </c>
       <c r="K77">
-        <v>57.3909499335277</v>
+        <v>62.6433899163336</v>
       </c>
       <c r="L77">
         <v>89.80584340279077</v>
@@ -4827,7 +4827,7 @@
         <v>27</v>
       </c>
       <c r="S77">
-        <v>31.21755793806243</v>
+        <v>25.96511795525653</v>
       </c>
     </row>
     <row r="78" spans="1:19">
@@ -7102,7 +7102,7 @@
         <v>0</v>
       </c>
       <c r="K118">
-        <v>61.48758237299869</v>
+        <v>57.85387248332849</v>
       </c>
       <c r="L118">
         <v>15.85204755614267</v>
@@ -7123,7 +7123,7 @@
         <v>24</v>
       </c>
       <c r="S118">
-        <v>-45.63553481685603</v>
+        <v>-42.00182492718583</v>
       </c>
     </row>
     <row r="119" spans="1:19">
@@ -7158,7 +7158,7 @@
         <v>0</v>
       </c>
       <c r="K119">
-        <v>61.48758237299869</v>
+        <v>57.85387248332849</v>
       </c>
       <c r="L119">
         <v>15.85204755614267</v>
@@ -7179,7 +7179,7 @@
         <v>25</v>
       </c>
       <c r="S119">
-        <v>-33.85444908186454</v>
+        <v>-30.22073919219433</v>
       </c>
     </row>
     <row r="120" spans="1:19">
@@ -7214,7 +7214,7 @@
         <v>0</v>
       </c>
       <c r="K120">
-        <v>61.48758237299869</v>
+        <v>57.85387248332849</v>
       </c>
       <c r="L120">
         <v>15.85204755614267</v>
@@ -7235,7 +7235,7 @@
         <v>26</v>
       </c>
       <c r="S120">
-        <v>-35.87001168407564</v>
+        <v>-32.23630179440543</v>
       </c>
     </row>
     <row r="121" spans="1:19">
@@ -7270,7 +7270,7 @@
         <v>0</v>
       </c>
       <c r="K121">
-        <v>61.48758237299869</v>
+        <v>57.85387248332849</v>
       </c>
       <c r="L121">
         <v>15.85204755614267</v>
@@ -7291,7 +7291,7 @@
         <v>27</v>
       </c>
       <c r="S121">
-        <v>-35.11721323032864</v>
+        <v>-31.48350334065845</v>
       </c>
     </row>
     <row r="122" spans="1:19">
@@ -9566,7 +9566,7 @@
         <v>0</v>
       </c>
       <c r="K162">
-        <v>53.9917012472936</v>
+        <v>58.9487860548799</v>
       </c>
       <c r="L162">
         <v>93.32799321490836</v>
@@ -9587,7 +9587,7 @@
         <v>24</v>
       </c>
       <c r="S162">
-        <v>39.33629196761476</v>
+        <v>34.37920716002846</v>
       </c>
     </row>
     <row r="163" spans="1:19">
@@ -9622,7 +9622,7 @@
         <v>0</v>
       </c>
       <c r="K163">
-        <v>53.9917012472936</v>
+        <v>58.9487860548799</v>
       </c>
       <c r="L163">
         <v>93.32799321490836</v>
@@ -9643,7 +9643,7 @@
         <v>25</v>
       </c>
       <c r="S163">
-        <v>40.93257833336629</v>
+        <v>35.97549352577999</v>
       </c>
     </row>
     <row r="164" spans="1:19">
@@ -9678,7 +9678,7 @@
         <v>0</v>
       </c>
       <c r="K164">
-        <v>53.9917012472936</v>
+        <v>58.9487860548799</v>
       </c>
       <c r="L164">
         <v>93.32799321490836</v>
@@ -9699,7 +9699,7 @@
         <v>26</v>
       </c>
       <c r="S164">
-        <v>36.87804756160919</v>
+        <v>31.9209627540229</v>
       </c>
     </row>
     <row r="165" spans="1:19">
@@ -9734,7 +9734,7 @@
         <v>0</v>
       </c>
       <c r="K165">
-        <v>53.9917012472936</v>
+        <v>58.9487860548799</v>
       </c>
       <c r="L165">
         <v>93.32799321490836</v>
@@ -9755,7 +9755,7 @@
         <v>27</v>
       </c>
       <c r="S165">
-        <v>36.82072060467674</v>
+        <v>31.86363579709044</v>
       </c>
     </row>
     <row r="166" spans="1:19">
@@ -12030,7 +12030,7 @@
         <v>1</v>
       </c>
       <c r="K206">
-        <v>66.13023562229581</v>
+        <v>63.06375972137231</v>
       </c>
       <c r="L206">
         <v>20.45869883040936</v>
@@ -12051,7 +12051,7 @@
         <v>24</v>
       </c>
       <c r="S206">
-        <v>-45.67153679188645</v>
+        <v>-42.60506089096295</v>
       </c>
     </row>
     <row r="207" spans="1:19">
@@ -12086,7 +12086,7 @@
         <v>1</v>
       </c>
       <c r="K207">
-        <v>66.13023562229581</v>
+        <v>63.06375972137231</v>
       </c>
       <c r="L207">
         <v>20.45869883040936</v>
@@ -12107,7 +12107,7 @@
         <v>25</v>
       </c>
       <c r="S207">
-        <v>-50.05777870600128</v>
+        <v>-46.99130280507777</v>
       </c>
     </row>
     <row r="208" spans="1:19">
@@ -12142,7 +12142,7 @@
         <v>1</v>
       </c>
       <c r="K208">
-        <v>66.13023562229581</v>
+        <v>63.06375972137231</v>
       </c>
       <c r="L208">
         <v>20.45869883040936</v>
@@ -12163,7 +12163,7 @@
         <v>26</v>
       </c>
       <c r="S208">
-        <v>-42.68873696686224</v>
+        <v>-39.62226106593874</v>
       </c>
     </row>
     <row r="209" spans="1:19">
@@ -12198,7 +12198,7 @@
         <v>1</v>
       </c>
       <c r="K209">
-        <v>66.13023562229581</v>
+        <v>63.06375972137231</v>
       </c>
       <c r="L209">
         <v>20.45869883040936</v>
@@ -12219,7 +12219,7 @@
         <v>27</v>
       </c>
       <c r="S209">
-        <v>-42.84433159538177</v>
+        <v>-39.77785569445827</v>
       </c>
     </row>
     <row r="210" spans="1:19">
@@ -14494,7 +14494,7 @@
         <v>1</v>
       </c>
       <c r="K250">
-        <v>55.4603219525063</v>
+        <v>60.45977516590651</v>
       </c>
       <c r="L250">
         <v>92.41490820524366</v>
@@ -14515,7 +14515,7 @@
         <v>24</v>
       </c>
       <c r="S250">
-        <v>36.95458625273736</v>
+        <v>31.95513303933716</v>
       </c>
     </row>
     <row r="251" spans="1:19">
@@ -14550,7 +14550,7 @@
         <v>1</v>
       </c>
       <c r="K251">
-        <v>55.4603219525063</v>
+        <v>60.45977516590651</v>
       </c>
       <c r="L251">
         <v>92.41490820524366</v>
@@ -14571,7 +14571,7 @@
         <v>25</v>
       </c>
       <c r="S251">
-        <v>37.99923351866112</v>
+        <v>32.99978030526092</v>
       </c>
     </row>
     <row r="252" spans="1:19">
@@ -14606,7 +14606,7 @@
         <v>1</v>
       </c>
       <c r="K252">
-        <v>55.4603219525063</v>
+        <v>60.45977516590651</v>
       </c>
       <c r="L252">
         <v>92.41490820524366</v>
@@ -14627,7 +14627,7 @@
         <v>26</v>
       </c>
       <c r="S252">
-        <v>36.39698451075576</v>
+        <v>31.39753129735555</v>
       </c>
     </row>
     <row r="253" spans="1:19">
@@ -14662,7 +14662,7 @@
         <v>1</v>
       </c>
       <c r="K253">
-        <v>55.4603219525063</v>
+        <v>60.45977516590651</v>
       </c>
       <c r="L253">
         <v>92.41490820524366</v>
@@ -14683,7 +14683,7 @@
         <v>27</v>
       </c>
       <c r="S253">
-        <v>36.54701397840824</v>
+        <v>31.54756076500803</v>
       </c>
     </row>
     <row r="254" spans="1:19">
@@ -16716,7 +16716,7 @@
         <v>43</v>
       </c>
       <c r="E290" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="F290" t="s">
         <v>46</v>
@@ -16734,19 +16734,19 @@
         <v>1</v>
       </c>
       <c r="K290">
-        <v>53.31034912579611</v>
+        <v>50.477072976542</v>
       </c>
       <c r="L290">
-        <v>11.78252784220314</v>
+        <v>88.21747215779686</v>
       </c>
       <c r="M290">
-        <v>16.02529247027256</v>
+        <v>83.97470752972744</v>
       </c>
       <c r="N290">
-        <v>11.48115825434971</v>
+        <v>88.51884174565029</v>
       </c>
       <c r="O290">
-        <v>11.76849713904182</v>
+        <v>88.23150286095819</v>
       </c>
       <c r="P290">
         <v>47859</v>
@@ -16755,7 +16755,7 @@
         <v>24</v>
       </c>
       <c r="S290">
-        <v>-41.52782128359297</v>
+        <v>37.74039918125486</v>
       </c>
     </row>
     <row r="291" spans="1:19">
@@ -16772,7 +16772,7 @@
         <v>43</v>
       </c>
       <c r="E291" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="F291" t="s">
         <v>46</v>
@@ -16790,19 +16790,19 @@
         <v>1</v>
       </c>
       <c r="K291">
-        <v>53.31034912579611</v>
+        <v>50.477072976542</v>
       </c>
       <c r="L291">
-        <v>11.78252784220314</v>
+        <v>88.21747215779686</v>
       </c>
       <c r="M291">
-        <v>16.02529247027256</v>
+        <v>83.97470752972744</v>
       </c>
       <c r="N291">
-        <v>11.48115825434971</v>
+        <v>88.51884174565029</v>
       </c>
       <c r="O291">
-        <v>11.76849713904182</v>
+        <v>88.23150286095819</v>
       </c>
       <c r="P291">
         <v>47859</v>
@@ -16811,7 +16811,7 @@
         <v>25</v>
       </c>
       <c r="S291">
-        <v>-37.28505665552355</v>
+        <v>33.49763455318543</v>
       </c>
     </row>
     <row r="292" spans="1:19">
@@ -16828,7 +16828,7 @@
         <v>43</v>
       </c>
       <c r="E292" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="F292" t="s">
         <v>46</v>
@@ -16846,19 +16846,19 @@
         <v>1</v>
       </c>
       <c r="K292">
-        <v>53.31034912579611</v>
+        <v>50.477072976542</v>
       </c>
       <c r="L292">
-        <v>11.78252784220314</v>
+        <v>88.21747215779686</v>
       </c>
       <c r="M292">
-        <v>16.02529247027256</v>
+        <v>83.97470752972744</v>
       </c>
       <c r="N292">
-        <v>11.48115825434971</v>
+        <v>88.51884174565029</v>
       </c>
       <c r="O292">
-        <v>11.76849713904182</v>
+        <v>88.23150286095819</v>
       </c>
       <c r="P292">
         <v>47859</v>
@@ -16867,7 +16867,7 @@
         <v>26</v>
       </c>
       <c r="S292">
-        <v>-41.8291908714464</v>
+        <v>38.04176876910829</v>
       </c>
     </row>
     <row r="293" spans="1:19">
@@ -16884,7 +16884,7 @@
         <v>43</v>
       </c>
       <c r="E293" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="F293" t="s">
         <v>46</v>
@@ -16902,19 +16902,19 @@
         <v>1</v>
       </c>
       <c r="K293">
-        <v>53.31034912579611</v>
+        <v>50.477072976542</v>
       </c>
       <c r="L293">
-        <v>11.78252784220314</v>
+        <v>88.21747215779686</v>
       </c>
       <c r="M293">
-        <v>16.02529247027256</v>
+        <v>83.97470752972744</v>
       </c>
       <c r="N293">
-        <v>11.48115825434971</v>
+        <v>88.51884174565029</v>
       </c>
       <c r="O293">
-        <v>11.76849713904182</v>
+        <v>88.23150286095819</v>
       </c>
       <c r="P293">
         <v>47859</v>
@@ -16923,7 +16923,7 @@
         <v>27</v>
       </c>
       <c r="S293">
-        <v>-41.54185198675429</v>
+        <v>37.75442988441618</v>
       </c>
     </row>
     <row r="294" spans="1:19">
@@ -19198,7 +19198,7 @@
         <v>1</v>
       </c>
       <c r="K334">
-        <v>61.6228045760042</v>
+        <v>66.6184922456773</v>
       </c>
       <c r="L334">
         <v>94.29505212642727</v>
@@ -19219,7 +19219,7 @@
         <v>24</v>
       </c>
       <c r="S334">
-        <v>32.67224755042307</v>
+        <v>27.67655988074997</v>
       </c>
     </row>
     <row r="335" spans="1:19">
@@ -19254,7 +19254,7 @@
         <v>1</v>
       </c>
       <c r="K335">
-        <v>61.6228045760042</v>
+        <v>66.6184922456773</v>
       </c>
       <c r="L335">
         <v>94.29505212642727</v>
@@ -19275,7 +19275,7 @@
         <v>25</v>
       </c>
       <c r="S335">
-        <v>28.74481469245583</v>
+        <v>23.74912702278273</v>
       </c>
     </row>
     <row r="336" spans="1:19">
@@ -19310,7 +19310,7 @@
         <v>1</v>
       </c>
       <c r="K336">
-        <v>61.6228045760042</v>
+        <v>66.6184922456773</v>
       </c>
       <c r="L336">
         <v>94.29505212642727</v>
@@ -19331,7 +19331,7 @@
         <v>26</v>
       </c>
       <c r="S336">
-        <v>33.03961575080498</v>
+        <v>28.04392808113188</v>
       </c>
     </row>
     <row r="337" spans="1:19">
@@ -19366,7 +19366,7 @@
         <v>1</v>
       </c>
       <c r="K337">
-        <v>61.6228045760042</v>
+        <v>66.6184922456773</v>
       </c>
       <c r="L337">
         <v>94.29505212642727</v>
@@ -19387,7 +19387,7 @@
         <v>27</v>
       </c>
       <c r="S337">
-        <v>33.16734853941211</v>
+        <v>28.17166086973901</v>
       </c>
     </row>
     <row r="338" spans="1:19">
@@ -21662,7 +21662,7 @@
         <v>0</v>
       </c>
       <c r="K378">
-        <v>57.0310306987091</v>
+        <v>53.51486207226939</v>
       </c>
       <c r="L378">
         <v>15.23428499612493</v>
@@ -21683,7 +21683,7 @@
         <v>24</v>
       </c>
       <c r="S378">
-        <v>-41.79674570258417</v>
+        <v>-38.28057707614447</v>
       </c>
     </row>
     <row r="379" spans="1:19">
@@ -21718,7 +21718,7 @@
         <v>0</v>
       </c>
       <c r="K379">
-        <v>57.0310306987091</v>
+        <v>53.51486207226939</v>
       </c>
       <c r="L379">
         <v>15.23428499612493</v>
@@ -21739,7 +21739,7 @@
         <v>25</v>
       </c>
       <c r="S379">
-        <v>-49.91344414536479</v>
+        <v>-46.3972755189251</v>
       </c>
     </row>
     <row r="380" spans="1:19">
@@ -21774,7 +21774,7 @@
         <v>0</v>
       </c>
       <c r="K380">
-        <v>57.0310306987091</v>
+        <v>53.51486207226939</v>
       </c>
       <c r="L380">
         <v>15.23428499612493</v>
@@ -21795,7 +21795,7 @@
         <v>26</v>
       </c>
       <c r="S380">
-        <v>-42.22879142349748</v>
+        <v>-38.71262279705778</v>
       </c>
     </row>
     <row r="381" spans="1:19">
@@ -21830,7 +21830,7 @@
         <v>0</v>
       </c>
       <c r="K381">
-        <v>57.0310306987091</v>
+        <v>53.51486207226939</v>
       </c>
       <c r="L381">
         <v>15.23428499612493</v>
@@ -21851,7 +21851,7 @@
         <v>27</v>
       </c>
       <c r="S381">
-        <v>-42.31245414533036</v>
+        <v>-38.79628551889066</v>
       </c>
     </row>
   </sheetData>

</xml_diff>